<commit_message>
Update codebase to latest version
</commit_message>
<xml_diff>
--- a/criminals/criminals.xlsx
+++ b/criminals/criminals.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -479,41 +479,41 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>usman_wilson</t>
+          <t>usman_khan</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>non-violent</t>
+          <t>property</t>
         </is>
       </c>
       <c r="G2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H2" t="b">
+        <v>1</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>bail</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>2018-07-30</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
         <v>6</v>
-      </c>
-      <c r="H2" t="b">
-        <v>0</v>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>parole</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>2024-08-15</t>
-        </is>
-      </c>
-      <c r="K2" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -522,41 +522,41 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>david_hassan</t>
+          <t>david_khan</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="n">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>fraud</t>
+          <t>sexual</t>
         </is>
       </c>
       <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="b">
         <v>0</v>
       </c>
-      <c r="H3" t="b">
-        <v>1</v>
-      </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>imprisoned</t>
+          <t>released</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2023-05-17</t>
+          <t>2019-09-22</t>
         </is>
       </c>
       <c r="K3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
@@ -565,12 +565,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ahmed_khan</t>
+          <t>ahmed_smith</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="n">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -586,7 +586,7 @@
         <v>6</v>
       </c>
       <c r="H4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -595,11 +595,11 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2018-10-24</t>
+          <t>2025-04-26</t>
         </is>
       </c>
       <c r="K4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -608,7 +608,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ivan_wilson</t>
+          <t>ivan_johnson</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -638,7 +638,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2021-03-23</t>
+          <t>2021-04-07</t>
         </is>
       </c>
       <c r="K5" t="n">
@@ -681,7 +681,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2022-06-11</t>
+          <t>2022-06-26</t>
         </is>
       </c>
       <c r="K6" t="n">
@@ -694,7 +694,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>yusuf_lee</t>
+          <t>yusuf_wilson</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -724,7 +724,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2018-10-27</t>
+          <t>2018-11-11</t>
         </is>
       </c>
       <c r="K7" t="n">
@@ -737,7 +737,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>elena_torres</t>
+          <t>elena_hassan</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -767,7 +767,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="K8" t="n">
@@ -780,7 +780,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>xena_lee</t>
+          <t>xena_khan</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -810,7 +810,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2019-02-07</t>
+          <t>2019-02-22</t>
         </is>
       </c>
       <c r="K9" t="n">
@@ -853,7 +853,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2023-01-16</t>
+          <t>2023-01-31</t>
         </is>
       </c>
       <c r="K10" t="n">
@@ -866,7 +866,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>nadia_ali</t>
+          <t>nadia_johnson</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -896,226 +896,11 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2020-04-04</t>
+          <t>2020-04-19</t>
         </is>
       </c>
       <c r="K11" t="n">
         <v>3</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>walter_johnson</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="n">
-        <v>21</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>drug</t>
-        </is>
-      </c>
-      <c r="G12" t="n">
-        <v>4</v>
-      </c>
-      <c r="H12" t="b">
-        <v>1</v>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>parole</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>2021-06-14</t>
-        </is>
-      </c>
-      <c r="K12" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>omar_petrov</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="n">
-        <v>51</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>property</t>
-        </is>
-      </c>
-      <c r="G13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" t="b">
-        <v>1</v>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>released</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>2019-01-09</t>
-        </is>
-      </c>
-      <c r="K13" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>bilal_hassan</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="n">
-        <v>43</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>fraud</t>
-        </is>
-      </c>
-      <c r="G14" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" t="b">
-        <v>1</v>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>imprisoned</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>2020-10-17</t>
-        </is>
-      </c>
-      <c r="K14" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>rania_malik</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="n">
-        <v>42</v>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>property</t>
-        </is>
-      </c>
-      <c r="G15" t="n">
-        <v>5</v>
-      </c>
-      <c r="H15" t="b">
-        <v>0</v>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>imprisoned</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>2024-08-19</t>
-        </is>
-      </c>
-      <c r="K15" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>layla_nguyen</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="n">
-        <v>51</v>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>fraud</t>
-        </is>
-      </c>
-      <c r="G16" t="n">
-        <v>7</v>
-      </c>
-      <c r="H16" t="b">
-        <v>1</v>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>wanted</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>2020-12-29</t>
-        </is>
-      </c>
-      <c r="K16" t="n">
-        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>